<commit_message>
Jose Francisco update 2
</commit_message>
<xml_diff>
--- a/data/raw/Copa_2026_2027/aggregate/aggregated_game_stats_with_defense.xlsx
+++ b/data/raw/Copa_2026_2027/aggregate/aggregated_game_stats_with_defense.xlsx
@@ -31821,7 +31821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW16"/>
+  <dimension ref="A1:AW15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33149,70 +33149,70 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="1" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P9" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S9" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T9" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="U9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="I9" s="1" t="n">
-        <v>4.666666666666667</v>
-      </c>
-      <c r="J9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="1" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="O9" s="1" t="n">
-        <v>1.666666666666667</v>
-      </c>
-      <c r="P9" s="1" t="n">
-        <v>1.666666666666667</v>
-      </c>
-      <c r="Q9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" s="1" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="T9" s="1" t="n">
-        <v>1.666666666666667</v>
-      </c>
-      <c r="U9" s="1" t="n">
-        <v>2.666666666666667</v>
-      </c>
       <c r="V9" s="1" t="n">
-        <v>5.333333333333333</v>
+        <v>5.75</v>
       </c>
       <c r="W9" s="1" t="n">
-        <v>50</v>
+        <v>52.17391304347826</v>
       </c>
       <c r="X9" s="1" t="n">
         <v>0</v>
@@ -33224,13 +33224,13 @@
         <v>0</v>
       </c>
       <c r="AA9" s="1" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.75</v>
       </c>
       <c r="AB9" s="1" t="n">
-        <v>0.6666666666666666</v>
+        <v>1.25</v>
       </c>
       <c r="AC9" s="1" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="AD9" s="1" t="n">
         <v>0</v>
@@ -33252,78 +33252,78 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:31</t>
         </is>
       </c>
       <c r="AK9" s="1" t="n">
-        <v>8.053333333333333</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AL9" s="1" t="n">
-        <v>50</v>
+        <v>53.57142857142857</v>
       </c>
       <c r="AM9" s="1" t="n">
-        <v>49.66887417218543</v>
+        <v>52.98913043478262</v>
       </c>
       <c r="AN9" s="1" t="n">
-        <v>0.823045267489712</v>
+        <v>0.9112149532710281</v>
       </c>
       <c r="AO9" s="1" t="n">
-        <v>17.14677640603567</v>
+        <v>14.01869158878505</v>
       </c>
       <c r="AP9" s="1" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="AQ9" s="1" t="n">
-        <v>18.26943177414965</v>
+        <v>20.09953797533571</v>
       </c>
       <c r="AR9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AS9" t="n">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="AT9" s="1" t="n">
-        <v>50</v>
+        <v>53.57142857142857</v>
       </c>
       <c r="AU9" s="1" t="n">
-        <v>50</v>
+        <v>53.57142857142857</v>
       </c>
       <c r="AV9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="AW9" s="1" t="n">
-        <v>42.85714285714285</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>#7 Jose López Martínez</t>
+          <t>#9 Eduard Illa Martinez</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>15</v>
+        <v>4.5</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>6</v>
+        <v>0.5</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>10</v>
+        <v>1.75</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="H10" s="1" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="I10" s="1" t="n">
-        <v>6</v>
+        <v>0.5</v>
       </c>
       <c r="J10" s="1" t="n">
         <v>0</v>
@@ -33338,145 +33338,145 @@
         <v>0</v>
       </c>
       <c r="N10" s="1" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="O10" s="1" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="P10" s="1" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="Q10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="1" t="n">
-        <v>7</v>
+        <v>1.25</v>
       </c>
       <c r="S10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="T10" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U10" s="1" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="V10" s="1" t="n">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="W10" s="1" t="n">
-        <v>57.14285714285714</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="Y10" s="1" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Z10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="AA10" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB10" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="1" t="n">
-        <v>66.66666666666666</v>
+        <v>0</v>
       </c>
       <c r="AD10" s="1" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="AE10" s="1" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AF10" s="1" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="AG10" s="1" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="AH10" s="1" t="n">
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="AI10" s="1" t="n">
-        <v>0</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>23:34</t>
+          <t>13:08</t>
         </is>
       </c>
       <c r="AK10" s="1" t="n">
-        <v>12.64</v>
+        <v>4.72</v>
       </c>
       <c r="AL10" s="1" t="n">
-        <v>60</v>
+        <v>44.44444444444444</v>
       </c>
       <c r="AM10" s="1" t="n">
-        <v>59.33544303797468</v>
+        <v>47.66949152542373</v>
       </c>
       <c r="AN10" s="1" t="n">
-        <v>1.099706744868035</v>
+        <v>0.9054325955734407</v>
       </c>
       <c r="AO10" s="1" t="n">
-        <v>7.331378299120233</v>
+        <v>5.030181086519115</v>
       </c>
       <c r="AP10" s="1" t="n">
-        <v>0.3</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="AQ10" s="1" t="n">
-        <v>25.57691381933813</v>
+        <v>16.71766385674717</v>
       </c>
       <c r="AR10" t="n">
-        <v>10</v>
+        <v>4.5</v>
       </c>
       <c r="AS10" t="n">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="AT10" s="1" t="n">
-        <v>60</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="AU10" s="1" t="n">
-        <v>60</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="AV10" s="1" t="n">
-        <v>0</v>
+        <v>36.36363636363637</v>
       </c>
       <c r="AW10" s="1" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>#9 Eduard Illa Martinez</t>
+          <t>#10 Xavi Maixenchs Bobe</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>1.75</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>0.5</v>
+        <v>2.333333333333333</v>
       </c>
       <c r="J11" s="1" t="n">
         <v>0</v>
@@ -33491,264 +33491,264 @@
         <v>0</v>
       </c>
       <c r="N11" s="1" t="n">
-        <v>0.25</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="O11" s="1" t="n">
-        <v>0.25</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="P11" s="1" t="n">
-        <v>0.75</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="Q11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="R11" s="1" t="n">
-        <v>1.25</v>
+        <v>-2.333333333333333</v>
       </c>
       <c r="S11" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T11" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U11" s="1" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="V11" s="1" t="n">
-        <v>1.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="W11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" s="1" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="AE11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF11" s="1" t="n">
         <v>33.33333333333333</v>
       </c>
-      <c r="X11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y11" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="Z11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD11" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AE11" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AF11" s="1" t="n">
-        <v>50</v>
-      </c>
       <c r="AG11" s="1" t="n">
-        <v>0.75</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="AH11" s="1" t="n">
-        <v>2.25</v>
+        <v>5</v>
       </c>
       <c r="AI11" s="1" t="n">
         <v>33.33333333333333</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>13:08</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="AK11" s="1" t="n">
-        <v>4.72</v>
+        <v>7.693333333333334</v>
       </c>
       <c r="AL11" s="1" t="n">
-        <v>44.44444444444444</v>
+        <v>45</v>
       </c>
       <c r="AM11" s="1" t="n">
-        <v>47.66949152542373</v>
+        <v>38.9948006932409</v>
       </c>
       <c r="AN11" s="1" t="n">
-        <v>0.9054325955734407</v>
+        <v>0.641025641025641</v>
       </c>
       <c r="AO11" s="1" t="n">
-        <v>5.030181086519115</v>
+        <v>17.8062678062678</v>
       </c>
       <c r="AP11" s="1" t="n">
-        <v>0.1111111111111111</v>
+        <v>0</v>
       </c>
       <c r="AQ11" s="1" t="n">
-        <v>16.71766385674717</v>
+        <v>25.00929492744666</v>
       </c>
       <c r="AR11" t="n">
-        <v>4.5</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="AS11" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="AT11" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AU11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV11" s="1" t="n">
         <v>33.33333333333333</v>
       </c>
-      <c r="AU11" s="1" t="n">
-        <v>28.57142857142857</v>
-      </c>
-      <c r="AV11" s="1" t="n">
-        <v>36.36363636363637</v>
-      </c>
       <c r="AW11" s="1" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>#10 Xavi Maixenchs Bobe</t>
+          <t>#12 Marc Latorre Rams</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="F12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="H12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="1" t="n">
-        <v>2.333333333333333</v>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="1" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="O12" s="1" t="n">
-        <v>1.666666666666667</v>
-      </c>
-      <c r="P12" s="1" t="n">
-        <v>1.666666666666667</v>
-      </c>
-      <c r="Q12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="1" t="n">
-        <v>-2.333333333333333</v>
-      </c>
-      <c r="S12" s="1" t="n">
+      <c r="U12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="X12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>03:07</t>
+        </is>
+      </c>
+      <c r="AK12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="T12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" s="1" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="W12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="1" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="AE12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF12" s="1" t="n">
-        <v>33.33333333333333</v>
-      </c>
-      <c r="AG12" s="1" t="n">
-        <v>1.666666666666667</v>
-      </c>
-      <c r="AH12" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="AI12" s="1" t="n">
-        <v>33.33333333333333</v>
-      </c>
-      <c r="AJ12" t="inlineStr">
-        <is>
-          <t>16:32</t>
-        </is>
-      </c>
-      <c r="AK12" s="1" t="n">
-        <v>7.693333333333334</v>
-      </c>
       <c r="AL12" s="1" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="AM12" s="1" t="n">
-        <v>38.9948006932409</v>
+        <v>50</v>
       </c>
       <c r="AN12" s="1" t="n">
-        <v>0.641025641025641</v>
+        <v>1</v>
       </c>
       <c r="AO12" s="1" t="n">
-        <v>17.8062678062678</v>
+        <v>0</v>
       </c>
       <c r="AP12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="AQ12" s="1" t="n">
-        <v>25.00929492744666</v>
+        <v>28.3577368705946</v>
       </c>
       <c r="AR12" t="n">
-        <v>6.666666666666667</v>
+        <v>2</v>
       </c>
       <c r="AS12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AT12" s="1" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="AU12" s="1" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AV12" s="1" t="n">
-        <v>33.33333333333333</v>
+        <v>0</v>
       </c>
       <c r="AW12" s="1" t="n">
         <v>0</v>
@@ -33757,185 +33757,185 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>#12 Marc Latorre Rams</t>
+          <t>#15 Joan Odena Massaguer</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C13" s="1" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="1" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="P13" s="1" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="Q13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="1" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="S13" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T13" s="1" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="U13" s="1" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="V13" s="1" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="W13" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="X13" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y13" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Z13" s="1" t="n">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="AA13" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AB13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="U13" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="V13" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="W13" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="X13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="AC13" s="1" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="AD13" s="1" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="AE13" s="1" t="n">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="AF13" s="1" t="n">
-        <v>0</v>
+        <v>9.090909090909092</v>
       </c>
       <c r="AG13" s="1" t="n">
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="AH13" s="1" t="n">
-        <v>1</v>
+        <v>5.5</v>
       </c>
       <c r="AI13" s="1" t="n">
-        <v>0</v>
+        <v>40.90909090909091</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>03:07</t>
+          <t>32:04</t>
         </is>
       </c>
       <c r="AK13" s="1" t="n">
-        <v>2</v>
+        <v>15.05</v>
       </c>
       <c r="AL13" s="1" t="n">
-        <v>50</v>
+        <v>51.72413793103448</v>
       </c>
       <c r="AM13" s="1" t="n">
-        <v>50</v>
+        <v>51.49501661129568</v>
       </c>
       <c r="AN13" s="1" t="n">
-        <v>1</v>
+        <v>0.950920245398773</v>
       </c>
       <c r="AO13" s="1" t="n">
-        <v>0</v>
+        <v>7.668711656441718</v>
       </c>
       <c r="AP13" s="1" t="n">
-        <v>0</v>
+        <v>0.03448275862068965</v>
       </c>
       <c r="AQ13" s="1" t="n">
-        <v>28.3577368705946</v>
+        <v>22.46289442704246</v>
       </c>
       <c r="AR13" t="n">
-        <v>2</v>
+        <v>14.5</v>
       </c>
       <c r="AS13" t="n">
-        <v>1</v>
+        <v>6.25</v>
       </c>
       <c r="AT13" s="1" t="n">
-        <v>50</v>
+        <v>43.10344827586206</v>
       </c>
       <c r="AU13" s="1" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="AV13" s="1" t="n">
-        <v>0</v>
+        <v>30.3030303030303</v>
       </c>
       <c r="AW13" s="1" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>#15 Joan Odena Massaguer</t>
+          <t>#17 Bru Postigo Camprubi</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>15.5</v>
+        <v>3.5</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>3.75</v>
+        <v>0.75</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>6.25</v>
+        <v>2.75</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>8.25</v>
+        <v>0.75</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>1.25</v>
+        <v>1.75</v>
       </c>
       <c r="J14" s="1" t="n">
         <v>0</v>
@@ -33950,419 +33950,266 @@
         <v>0</v>
       </c>
       <c r="N14" s="1" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="O14" s="1" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="P14" s="1" t="n">
-        <v>2.25</v>
+        <v>0.5</v>
       </c>
       <c r="Q14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="R14" s="1" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="S14" s="1" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="T14" s="1" t="n">
-        <v>5.25</v>
+        <v>0.5</v>
       </c>
       <c r="U14" s="1" t="n">
-        <v>1.75</v>
+        <v>0.5</v>
       </c>
       <c r="V14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="W14" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="X14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AB14" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AC14" s="1" t="n">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="AD14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AF14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AH14" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AI14" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="AK14" s="1" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="AL14" s="1" t="n">
+        <v>32.14285714285715</v>
+      </c>
+      <c r="AM14" s="1" t="n">
+        <v>40.98360655737706</v>
+      </c>
+      <c r="AN14" s="1" t="n">
+        <v>0.6972111553784861</v>
+      </c>
+      <c r="AO14" s="1" t="n">
+        <v>14.9402390438247</v>
+      </c>
+      <c r="AP14" s="1" t="n">
+        <v>0.3571428571428572</v>
+      </c>
+      <c r="AQ14" s="1" t="n">
+        <v>14.79329919972324</v>
+      </c>
+      <c r="AR14" t="n">
         <v>3.5</v>
       </c>
-      <c r="W14" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="X14" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Y14" s="1" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="Z14" s="1" t="n">
-        <v>66.66666666666666</v>
-      </c>
-      <c r="AA14" s="1" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AB14" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC14" s="1" t="n">
-        <v>75</v>
-      </c>
-      <c r="AD14" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AE14" s="1" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="AF14" s="1" t="n">
-        <v>9.090909090909092</v>
-      </c>
-      <c r="AG14" s="1" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="AH14" s="1" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="AI14" s="1" t="n">
-        <v>40.90909090909091</v>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>32:04</t>
-        </is>
-      </c>
-      <c r="AK14" s="1" t="n">
-        <v>15.05</v>
-      </c>
-      <c r="AL14" s="1" t="n">
-        <v>51.72413793103448</v>
-      </c>
-      <c r="AM14" s="1" t="n">
-        <v>51.49501661129568</v>
-      </c>
-      <c r="AN14" s="1" t="n">
-        <v>0.950920245398773</v>
-      </c>
-      <c r="AO14" s="1" t="n">
-        <v>7.668711656441718</v>
-      </c>
-      <c r="AP14" s="1" t="n">
-        <v>0.03448275862068965</v>
-      </c>
-      <c r="AQ14" s="1" t="n">
-        <v>22.46289442704246</v>
-      </c>
-      <c r="AR14" t="n">
-        <v>14.5</v>
-      </c>
       <c r="AS14" t="n">
-        <v>6.25</v>
+        <v>1</v>
       </c>
       <c r="AT14" s="1" t="n">
-        <v>43.10344827586206</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="AU14" s="1" t="n">
-        <v>60</v>
+        <v>27.27272727272727</v>
       </c>
       <c r="AV14" s="1" t="n">
-        <v>30.3030303030303</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="AW14" s="1" t="n">
-        <v>40</v>
+        <v>71.42857142857143</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>#17 Bru Postigo Camprubi</t>
+          <t>#28 Iago Carbajo Aubeso</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
         <v>4</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>3.5</v>
+        <v>1.75</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>0.75</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>2.75</v>
+        <v>1.75</v>
       </c>
       <c r="F15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1" t="n">
         <v>0.25</v>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="I15" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" s="1" t="n">
         <v>0.75</v>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="Q15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="1" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="S15" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T15" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U15" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V15" s="1" t="n">
         <v>1.25</v>
       </c>
-      <c r="I15" s="1" t="n">
+      <c r="W15" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="X15" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Y15" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Z15" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="AK15" s="1" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="AL15" s="1" t="n">
+        <v>42.85714285714285</v>
+      </c>
+      <c r="AM15" s="1" t="n">
+        <v>44.41624365482234</v>
+      </c>
+      <c r="AN15" s="1" t="n">
+        <v>0.5892255892255893</v>
+      </c>
+      <c r="AO15" s="1" t="n">
+        <v>33.67003367003367</v>
+      </c>
+      <c r="AP15" s="1" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="AQ15" s="1" t="n">
+        <v>11.277911550705</v>
+      </c>
+      <c r="AR15" t="n">
         <v>1.75</v>
       </c>
-      <c r="J15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O15" s="1" t="n">
+      <c r="AS15" t="n">
         <v>0.75</v>
       </c>
-      <c r="P15" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="T15" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="U15" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="V15" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="W15" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="X15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA15" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AB15" s="1" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AC15" s="1" t="n">
-        <v>33.33333333333333</v>
-      </c>
-      <c r="AD15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE15" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AF15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG15" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AH15" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AI15" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>14:59</t>
-        </is>
-      </c>
-      <c r="AK15" s="1" t="n">
-        <v>4.27</v>
-      </c>
-      <c r="AL15" s="1" t="n">
-        <v>32.14285714285715</v>
-      </c>
-      <c r="AM15" s="1" t="n">
-        <v>40.98360655737706</v>
-      </c>
-      <c r="AN15" s="1" t="n">
-        <v>0.6972111553784861</v>
-      </c>
-      <c r="AO15" s="1" t="n">
-        <v>14.9402390438247</v>
-      </c>
-      <c r="AP15" s="1" t="n">
-        <v>0.3571428571428572</v>
-      </c>
-      <c r="AQ15" s="1" t="n">
-        <v>14.79329919972324</v>
-      </c>
-      <c r="AR15" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="AS15" t="n">
-        <v>1</v>
-      </c>
       <c r="AT15" s="1" t="n">
-        <v>28.57142857142857</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="AU15" s="1" t="n">
-        <v>27.27272727272727</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="AV15" s="1" t="n">
-        <v>33.33333333333333</v>
+        <v>0</v>
       </c>
       <c r="AW15" s="1" t="n">
-        <v>71.42857142857143</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>#28 Iago Carbajo Aubeso</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C16" s="1" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="D16" s="1" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E16" s="1" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="F16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="I16" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" s="1" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="Q16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="1" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="S16" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T16" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="U16" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="V16" s="1" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="W16" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="X16" s="1" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="Y16" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Z16" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="AA16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ16" t="inlineStr">
-        <is>
-          <t>11:38</t>
-        </is>
-      </c>
-      <c r="AK16" s="1" t="n">
-        <v>1.97</v>
-      </c>
-      <c r="AL16" s="1" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="AM16" s="1" t="n">
-        <v>44.41624365482234</v>
-      </c>
-      <c r="AN16" s="1" t="n">
-        <v>0.5892255892255893</v>
-      </c>
-      <c r="AO16" s="1" t="n">
-        <v>33.67003367003367</v>
-      </c>
-      <c r="AP16" s="1" t="n">
-        <v>0.1428571428571428</v>
-      </c>
-      <c r="AQ16" s="1" t="n">
-        <v>11.277911550705</v>
-      </c>
-      <c r="AR16" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="AS16" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="AT16" s="1" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="AU16" s="1" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="AV16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW16" s="1" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>